<commit_message>
fix: stabilize mobile dock navigation and actions menu4
</commit_message>
<xml_diff>
--- a/reyes_monitoreo_base_v1.xlsx
+++ b/reyes_monitoreo_base_v1.xlsx
@@ -14713,7 +14713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14841,198 +14841,6 @@
         <is>
           <t>alerta</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SI/NO</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>copiar desde PRODUCTOS_REYES</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>copiar desde PRODUCTOS_REYES</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>REDLENIC o IMPOTEKNO</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>pegar link de categoría</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>texto para ubicar el producto en la web</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>si el sitio muestra código</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>si existe una imagen o link de imagen</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>traer de CONFIG</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>lo completa el sistema</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>OK / NO ENCONTRADO / ERROR</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>mensaje corto</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>12345</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Pava eléctrica negra 1.8L</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>REDLENIC</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.redlenic.uno/catalogo2024.php?rub=18#productos</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>pava eléctrica negra</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>42</v>
-      </c>
-      <c r="J3" t="n">
-        <v>42</v>
-      </c>
-      <c r="K3" t="n">
-        <v>18</v>
-      </c>
-      <c r="N3" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="R3" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>67890</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Auricular bluetooth rosa</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>IMPOTEKNO</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://impotekno.com/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>auricular rosa bluetooth</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>29990</v>
-      </c>
-      <c r="J4" t="n">
-        <v>14</v>
-      </c>
-      <c r="K4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N4" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="R4" t="n">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -15074,7 +14882,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1430.0</t>
+          <t>1400.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -15187,7 +14995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15243,8 +15051,6 @@
           <t>CAMBIO_CONFIG</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>dolar_oficial</t>
@@ -15309,8 +15115,6 @@
           <t>CAMBIO_CONFIG</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>dolar_oficial</t>
@@ -15339,8 +15143,6 @@
           <t>CAMBIO_CONFIG</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>dolar_blue</t>
@@ -15369,8 +15171,6 @@
           <t>CAMBIO_CONFIG</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>dolar_modo</t>
@@ -15387,6 +15187,38 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-21 21:31:48</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CAMBIO_CONFIG</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>dolar_oficial</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1430</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>sistema</t>
         </is>

</xml_diff>